<commit_message>
docs(certification): dossier, annexes et support de formation Bloc 2 (RNCP 39586)
Bloc 2 — Analyser, organiser et valoriser des données (8 compétences) :
- dossier écrit (C2.1.1 → C2.3.2) avec captures dashboard intégrées
- annexes A-H (captures Vue d'ensemble / Coûts&ROI / Test du modèle,
  rapport des 4 tests statistiques, dictionnaire des indicateurs)
- support de formation (public non technique, 6 modules)
- rapport des tests d'hypothèses + captures d'écran
</commit_message>
<xml_diff>
--- a/docs/certification/Bloc 1/#11 domain_model_run9.xlsx
+++ b/docs/certification/Bloc 1/#11 domain_model_run9.xlsx
@@ -1180,10 +1180,10 @@
         <v>2.1629</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>2.1629</v>
+        <v>1.6611</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>0</v>
@@ -1208,10 +1208,10 @@
         <v>1.8451</v>
       </c>
       <c r="F3" t="n">
-        <v>1.8451</v>
+        <v>1.4171</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1236,10 +1236,10 @@
         <v>0.1522</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.1522</v>
+        <v>0.1169</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0</v>
+        <v>-0.04</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>0</v>
@@ -1264,10 +1264,10 @@
         <v>0.1323</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1323</v>
+        <v>0.1016</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>-0.03</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -1292,7 +1292,7 @@
         <v>0.0124</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.0124</v>
+        <v>0.0095</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>0.009599999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0073</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1348,7 +1348,7 @@
         <v>0.006</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.006</v>
+        <v>0.0046</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0.0052</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0052</v>
+        <v>0.004</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1471,22 +1471,22 @@
         <v>7.8366</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2.16</v>
+        <v>1.66</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>7.8366</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.66</v>
+        <v>0.4</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.51</v>
+        <v>1.26</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1.51</v>
+        <v>1.26</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.51</v>
+        <v>1.26</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>1</v>
@@ -1503,22 +1503,22 @@
         <v>9.003299999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>4.65</v>
+        <v>3.57</v>
       </c>
       <c r="D3" t="n">
         <v>8.5116</v>
       </c>
       <c r="E3" t="n">
-        <v>1.39</v>
+        <v>0.86</v>
       </c>
       <c r="F3" t="n">
-        <v>3.15</v>
+        <v>2.62</v>
       </c>
       <c r="G3" t="n">
-        <v>3.26</v>
+        <v>2.71</v>
       </c>
       <c r="H3" t="n">
-        <v>3.36</v>
+        <v>2.8</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
@@ -1535,22 +1535,22 @@
         <v>10.3437</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.5</v>
+        <v>5.76</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>9.250500000000001</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.2</v>
+        <v>1.37</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>4.94</v>
+        <v>4.11</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>5.3</v>
+        <v>4.4</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>5.65</v>
+        <v>4.68</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>1</v>
@@ -1567,22 +1567,22 @@
         <v>11.8836</v>
       </c>
       <c r="C5" t="n">
-        <v>10.78</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D5" t="n">
         <v>10.0601</v>
       </c>
       <c r="E5" t="n">
-        <v>3.11</v>
+        <v>1.94</v>
       </c>
       <c r="F5" t="n">
-        <v>6.88</v>
+        <v>5.72</v>
       </c>
       <c r="G5" t="n">
-        <v>7.67</v>
+        <v>6.34</v>
       </c>
       <c r="H5" t="n">
-        <v>8.460000000000001</v>
+        <v>6.97</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -1599,22 +1599,22 @@
         <v>13.6528</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>14.55</v>
+        <v>11.17</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>10.9479</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>4.13</v>
+        <v>2.58</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>9</v>
+        <v>7.46</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>10.42</v>
+        <v>8.59</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>11.91</v>
+        <v>9.77</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>1</v>
@@ -1631,22 +1631,22 @@
         <v>15.6854</v>
       </c>
       <c r="C7" t="n">
-        <v>18.88</v>
+        <v>14.5</v>
       </c>
       <c r="D7" t="n">
         <v>11.9226</v>
       </c>
       <c r="E7" t="n">
-        <v>5.26</v>
+        <v>3.31</v>
       </c>
       <c r="F7" t="n">
-        <v>11.31</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>13.62</v>
+        <v>11.19</v>
       </c>
       <c r="H7" t="n">
-        <v>16.14</v>
+        <v>13.19</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-14T22:49:08</t>
+          <t>2026-07-17T15:46:42</t>
         </is>
       </c>
     </row>
@@ -20111,22 +20111,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CONSERVATION_REGLEMENTAIRE</t>
+          <t>CONSERVATION_SECURISEE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Conservation réglementaire</t>
+          <t>Conservation sécurisée</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Donnée d'un domaine réglementé (Finance, RH, Achats, Ventes) encore dans sa fenêtre de rétention légale.</t>
+          <t>Données personnelles (PII) actives ou récentes.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Conserver en stockage actif jusqu'à expiration de la rétention légale du domaine. Ne pas archiver à froid ni purger (risque de non-conformité). Réévaluer ensuite.</t>
+          <t>Conserver en stockage actif avec contrôle d'accès renforcé et journalisation.</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -20136,22 +20136,22 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CONSERVATION_SECURISEE</t>
+          <t>CONSERVATION_REGLEMENTAIRE</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Conservation sécurisée</t>
+          <t>Conservation réglementaire</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Données personnelles (PII) actives ou récentes.</t>
+          <t>Donnée d'un domaine réglementé (Finance, RH, Achats, Ventes) encore dans sa fenêtre de rétention légale.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Conserver en stockage actif avec contrôle d'accès renforcé et journalisation.</t>
+          <t>Conserver en stockage actif jusqu'à expiration de la rétention légale du domaine. Ne pas archiver à froid ni purger (risque de non-conformité). Réévaluer ensuite.</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
@@ -64607,7 +64607,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>0.276</v>
+        <v>0.211968</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -64627,7 +64627,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.048</v>
+        <v>0.0216</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -64802,19 +64802,19 @@
         <v>6.6853</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1.85</v>
+        <v>1.42</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>1.42</v>
+        <v>1.18</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>76.8</v>
+        <v>83.5</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>85.25</v>
+        <v>85.54000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>85.3</v>
+        <v>85.5</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>1</v>
@@ -64835,19 +64835,19 @@
         <v>0.5515</v>
       </c>
       <c r="C3" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="F3" t="n">
-        <v>6.91</v>
+        <v>7.23</v>
       </c>
       <c r="G3" t="n">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="H3" t="n">
         <v>2</v>
@@ -64868,19 +64868,19 @@
         <v>0.4794</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>58.5</v>
+        <v>63.6</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>5.99</v>
+        <v>6.02</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>98.2</v>
+        <v>98.8</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>3</v>
@@ -64907,13 +64907,13 @@
         <v>0.01</v>
       </c>
       <c r="E5" t="n">
-        <v>49.5</v>
+        <v>53.8</v>
       </c>
       <c r="F5" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
       <c r="G5" t="n">
-        <v>98.59999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="H5" t="n">
         <v>4</v>
@@ -64927,11 +64927,11 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Ventes &amp; Clients</t>
+          <t>Achats &amp; Fournisseurs</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.019</v>
+        <v>0.0347</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>0.01</v>
@@ -64940,13 +64940,13 @@
         <v>0</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>4</v>
@@ -64960,66 +64960,66 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Ventes &amp; Clients</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0218</v>
+        <v>0.019</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>32.6</v>
+        <v>2.9</v>
       </c>
       <c r="F7" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Faible</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Achats &amp; Fournisseurs</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0.0347</v>
+        <v>0.0218</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>8.5</v>
+        <v>35.5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Élevé</t>
         </is>
       </c>
     </row>

</xml_diff>